<commit_message>
Update: Problematica y Datos (Informe)
</commit_message>
<xml_diff>
--- a/F-SST-015 Inspeccion  Vehiculo  GRUA MANLIFT.xlsx
+++ b/F-SST-015 Inspeccion  Vehiculo  GRUA MANLIFT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://americanlightingcom-my.sharepoint.com/personal/supervisorhseqzona3_americanlightingsas_com/Documents/Escritorio/2024/4.FORMATOS/FORMATOS SEMANALES AML/MANTENIMIENTO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XJuan\source\repos\AutoCheckAML\Docs-AutoCheck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{26015F93-395B-4377-BEB3-FB3F9619D744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10D7438B-38EE-4BF9-B6A3-EF8FD794C2D0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1D101E-5967-40A4-A3F1-5A000646CD32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -33,9 +33,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -274,9 +271,6 @@
     <t>Version: 01</t>
   </si>
   <si>
-    <t>Fecha: 05-04-2016</t>
-  </si>
-  <si>
     <t>Pagina 1 de 1</t>
   </si>
   <si>
@@ -305,6 +299,9 @@
   </si>
   <si>
     <t>FIRMA DEL CONDUCTOR:</t>
+  </si>
+  <si>
+    <t>Fecha: 12-06-2026</t>
   </si>
 </sst>
 </file>
@@ -1109,275 +1106,275 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1463,13 +1460,13 @@
           <xdr:col>15</xdr:col>
           <xdr:colOff>533400</xdr:colOff>
           <xdr:row>20</xdr:row>
-          <xdr:rowOff>180975</xdr:rowOff>
+          <xdr:rowOff>182880</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>17</xdr:col>
-          <xdr:colOff>466725</xdr:colOff>
+          <xdr:colOff>464820</xdr:colOff>
           <xdr:row>31</xdr:row>
-          <xdr:rowOff>95250</xdr:rowOff>
+          <xdr:rowOff>99060</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1515,15 +1512,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>47625</xdr:colOff>
+          <xdr:colOff>45720</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>57150</xdr:rowOff>
+          <xdr:rowOff>60960</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>1400175</xdr:colOff>
+          <xdr:colOff>1402080</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>2000250</xdr:rowOff>
+          <xdr:rowOff>2004060</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1569,9 +1566,9 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>66675</xdr:colOff>
+          <xdr:colOff>68580</xdr:colOff>
           <xdr:row>2</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>106680</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
@@ -1623,15 +1620,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>95250</xdr:colOff>
+          <xdr:colOff>99060</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>85725</xdr:rowOff>
+          <xdr:rowOff>83820</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>1419225</xdr:colOff>
+          <xdr:colOff>1417320</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>2000250</xdr:rowOff>
+          <xdr:rowOff>2004060</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1677,15 +1674,15 @@
       <xdr:twoCellAnchor>
         <xdr:from>
           <xdr:col>0</xdr:col>
-          <xdr:colOff>133350</xdr:colOff>
+          <xdr:colOff>137160</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>47625</xdr:rowOff>
+          <xdr:rowOff>45720</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>0</xdr:col>
           <xdr:colOff>1485900</xdr:colOff>
           <xdr:row>4</xdr:row>
-          <xdr:rowOff>2000250</xdr:rowOff>
+          <xdr:rowOff>2004060</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2057,369 +2054,369 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" customWidth="1"/>
-    <col min="4" max="4" width="4.28515625" style="34" customWidth="1"/>
-    <col min="5" max="5" width="4.28515625" customWidth="1"/>
-    <col min="6" max="9" width="4.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="4.33203125" style="34" customWidth="1"/>
+    <col min="5" max="5" width="4.33203125" customWidth="1"/>
+    <col min="6" max="9" width="4.88671875" customWidth="1"/>
     <col min="10" max="11" width="5" customWidth="1"/>
-    <col min="12" max="13" width="5.42578125" customWidth="1"/>
-    <col min="14" max="15" width="5.28515625" customWidth="1"/>
-    <col min="16" max="16" width="27.42578125" customWidth="1"/>
-    <col min="19" max="19" width="22.140625" customWidth="1"/>
+    <col min="12" max="13" width="5.44140625" customWidth="1"/>
+    <col min="14" max="15" width="5.33203125" customWidth="1"/>
+    <col min="16" max="16" width="27.44140625" customWidth="1"/>
+    <col min="19" max="19" width="22.109375" customWidth="1"/>
     <col min="20" max="21" width="5" customWidth="1"/>
-    <col min="22" max="23" width="5.28515625" customWidth="1"/>
+    <col min="22" max="23" width="5.33203125" customWidth="1"/>
     <col min="24" max="25" width="5" customWidth="1"/>
-    <col min="26" max="27" width="4.85546875" customWidth="1"/>
-    <col min="28" max="29" width="4.42578125" customWidth="1"/>
-    <col min="30" max="31" width="4.85546875" customWidth="1"/>
-    <col min="32" max="32" width="25.7109375" customWidth="1"/>
+    <col min="26" max="27" width="4.88671875" customWidth="1"/>
+    <col min="28" max="29" width="4.44140625" customWidth="1"/>
+    <col min="30" max="31" width="4.88671875" customWidth="1"/>
+    <col min="32" max="32" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="51"/>
+      <c r="Y1" s="51"/>
+      <c r="Z1" s="52"/>
+      <c r="AA1" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="122"/>
-      <c r="F1" s="122"/>
-      <c r="G1" s="122"/>
-      <c r="H1" s="122"/>
-      <c r="I1" s="122"/>
-      <c r="J1" s="122"/>
-      <c r="K1" s="122"/>
-      <c r="L1" s="122"/>
-      <c r="M1" s="122"/>
-      <c r="N1" s="122"/>
-      <c r="O1" s="122"/>
-      <c r="P1" s="122"/>
-      <c r="Q1" s="122"/>
-      <c r="R1" s="122"/>
-      <c r="S1" s="122"/>
-      <c r="T1" s="122"/>
-      <c r="U1" s="122"/>
-      <c r="V1" s="122"/>
-      <c r="W1" s="122"/>
-      <c r="X1" s="122"/>
-      <c r="Y1" s="122"/>
-      <c r="Z1" s="123"/>
-      <c r="AA1" s="130" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB1" s="131"/>
-      <c r="AC1" s="131"/>
-      <c r="AD1" s="131"/>
-      <c r="AE1" s="131"/>
-      <c r="AF1" s="132"/>
-    </row>
-    <row r="2" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="124"/>
-      <c r="B2" s="125"/>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="125"/>
-      <c r="J2" s="125"/>
-      <c r="K2" s="125"/>
-      <c r="L2" s="125"/>
-      <c r="M2" s="125"/>
-      <c r="N2" s="125"/>
-      <c r="O2" s="125"/>
-      <c r="P2" s="125"/>
-      <c r="Q2" s="125"/>
-      <c r="R2" s="125"/>
-      <c r="S2" s="125"/>
-      <c r="T2" s="125"/>
-      <c r="U2" s="125"/>
-      <c r="V2" s="125"/>
-      <c r="W2" s="125"/>
-      <c r="X2" s="125"/>
-      <c r="Y2" s="125"/>
-      <c r="Z2" s="126"/>
-      <c r="AA2" s="121"/>
-      <c r="AB2" s="122"/>
-      <c r="AC2" s="122"/>
-      <c r="AD2" s="122"/>
-      <c r="AE2" s="123"/>
+      <c r="AB1" s="60"/>
+      <c r="AC1" s="60"/>
+      <c r="AD1" s="60"/>
+      <c r="AE1" s="60"/>
+      <c r="AF1" s="61"/>
+    </row>
+    <row r="2" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="53"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="Q2" s="54"/>
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
+      <c r="V2" s="54"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="54"/>
+      <c r="Y2" s="54"/>
+      <c r="Z2" s="55"/>
+      <c r="AA2" s="50"/>
+      <c r="AB2" s="51"/>
+      <c r="AC2" s="51"/>
+      <c r="AD2" s="51"/>
+      <c r="AE2" s="52"/>
       <c r="AF2" s="26" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="124"/>
-      <c r="B3" s="125"/>
-      <c r="C3" s="125"/>
-      <c r="D3" s="125"/>
-      <c r="E3" s="125"/>
-      <c r="F3" s="125"/>
-      <c r="G3" s="125"/>
-      <c r="H3" s="125"/>
-      <c r="I3" s="125"/>
-      <c r="J3" s="125"/>
-      <c r="K3" s="125"/>
-      <c r="L3" s="125"/>
-      <c r="M3" s="125"/>
-      <c r="N3" s="125"/>
-      <c r="O3" s="125"/>
-      <c r="P3" s="125"/>
-      <c r="Q3" s="125"/>
-      <c r="R3" s="125"/>
-      <c r="S3" s="125"/>
-      <c r="T3" s="125"/>
-      <c r="U3" s="125"/>
-      <c r="V3" s="125"/>
-      <c r="W3" s="125"/>
-      <c r="X3" s="125"/>
-      <c r="Y3" s="125"/>
-      <c r="Z3" s="126"/>
-      <c r="AA3" s="124"/>
-      <c r="AB3" s="125"/>
-      <c r="AC3" s="125"/>
-      <c r="AD3" s="125"/>
-      <c r="AE3" s="126"/>
+    <row r="3" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="53"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54"/>
+      <c r="U3" s="54"/>
+      <c r="V3" s="54"/>
+      <c r="W3" s="54"/>
+      <c r="X3" s="54"/>
+      <c r="Y3" s="54"/>
+      <c r="Z3" s="55"/>
+      <c r="AA3" s="53"/>
+      <c r="AB3" s="54"/>
+      <c r="AC3" s="54"/>
+      <c r="AD3" s="54"/>
+      <c r="AE3" s="55"/>
       <c r="AF3" s="26" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="56"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="57"/>
+      <c r="N4" s="57"/>
+      <c r="O4" s="57"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="57"/>
+      <c r="R4" s="57"/>
+      <c r="S4" s="57"/>
+      <c r="T4" s="57"/>
+      <c r="U4" s="57"/>
+      <c r="V4" s="57"/>
+      <c r="W4" s="57"/>
+      <c r="X4" s="57"/>
+      <c r="Y4" s="57"/>
+      <c r="Z4" s="58"/>
+      <c r="AA4" s="56"/>
+      <c r="AB4" s="57"/>
+      <c r="AC4" s="57"/>
+      <c r="AD4" s="57"/>
+      <c r="AE4" s="58"/>
+      <c r="AF4" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:32" s="7" customFormat="1" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="127"/>
-      <c r="B4" s="128"/>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128"/>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128"/>
-      <c r="G4" s="128"/>
-      <c r="H4" s="128"/>
-      <c r="I4" s="128"/>
-      <c r="J4" s="128"/>
-      <c r="K4" s="128"/>
-      <c r="L4" s="128"/>
-      <c r="M4" s="128"/>
-      <c r="N4" s="128"/>
-      <c r="O4" s="128"/>
-      <c r="P4" s="128"/>
-      <c r="Q4" s="128"/>
-      <c r="R4" s="128"/>
-      <c r="S4" s="128"/>
-      <c r="T4" s="128"/>
-      <c r="U4" s="128"/>
-      <c r="V4" s="128"/>
-      <c r="W4" s="128"/>
-      <c r="X4" s="128"/>
-      <c r="Y4" s="128"/>
-      <c r="Z4" s="129"/>
-      <c r="AA4" s="127"/>
-      <c r="AB4" s="128"/>
-      <c r="AC4" s="128"/>
-      <c r="AD4" s="128"/>
-      <c r="AE4" s="129"/>
-      <c r="AF4" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:32" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="73" t="s">
+    <row r="5" spans="1:32" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="109" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74"/>
-      <c r="J5" s="74"/>
-      <c r="K5" s="74"/>
-      <c r="L5" s="74"/>
-      <c r="M5" s="74"/>
-      <c r="N5" s="74"/>
-      <c r="O5" s="74"/>
-      <c r="P5" s="75"/>
-      <c r="Q5" s="73" t="s">
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
+      <c r="O5" s="68"/>
+      <c r="P5" s="95"/>
+      <c r="Q5" s="109" t="s">
         <v>1</v>
       </c>
-      <c r="R5" s="74"/>
-      <c r="S5" s="74"/>
-      <c r="T5" s="74"/>
-      <c r="U5" s="74"/>
-      <c r="V5" s="74"/>
-      <c r="W5" s="74"/>
-      <c r="X5" s="74"/>
-      <c r="Y5" s="74"/>
-      <c r="Z5" s="74"/>
-      <c r="AA5" s="74"/>
-      <c r="AB5" s="74"/>
-      <c r="AC5" s="74"/>
-      <c r="AD5" s="74"/>
-      <c r="AE5" s="74"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="68"/>
+      <c r="Y5" s="68"/>
+      <c r="Z5" s="68"/>
+      <c r="AA5" s="68"/>
+      <c r="AB5" s="68"/>
+      <c r="AC5" s="68"/>
+      <c r="AD5" s="68"/>
+      <c r="AE5" s="68"/>
       <c r="AF5" s="8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:32" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="99" t="s">
+    <row r="6" spans="1:32" s="7" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="125" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="99"/>
-      <c r="C6" s="71"/>
-      <c r="D6" s="71"/>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="71"/>
-      <c r="M6" s="71"/>
-      <c r="N6" s="71"/>
-      <c r="O6" s="72"/>
+      <c r="B6" s="125"/>
+      <c r="C6" s="107"/>
+      <c r="D6" s="107"/>
+      <c r="E6" s="107"/>
+      <c r="F6" s="107"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="107"/>
+      <c r="I6" s="107"/>
+      <c r="J6" s="107"/>
+      <c r="K6" s="107"/>
+      <c r="L6" s="107"/>
+      <c r="M6" s="107"/>
+      <c r="N6" s="107"/>
+      <c r="O6" s="108"/>
       <c r="P6" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="Q6" s="73" t="s">
+      <c r="Q6" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="R6" s="74"/>
-      <c r="S6" s="74"/>
-      <c r="T6" s="74"/>
-      <c r="U6" s="74"/>
-      <c r="V6" s="74"/>
-      <c r="W6" s="74"/>
-      <c r="X6" s="74"/>
-      <c r="Y6" s="74"/>
-      <c r="Z6" s="74"/>
-      <c r="AA6" s="74"/>
-      <c r="AB6" s="74"/>
-      <c r="AC6" s="74"/>
-      <c r="AD6" s="74"/>
-      <c r="AE6" s="74"/>
+      <c r="R6" s="68"/>
+      <c r="S6" s="68"/>
+      <c r="T6" s="68"/>
+      <c r="U6" s="68"/>
+      <c r="V6" s="68"/>
+      <c r="W6" s="68"/>
+      <c r="X6" s="68"/>
+      <c r="Y6" s="68"/>
+      <c r="Z6" s="68"/>
+      <c r="AA6" s="68"/>
+      <c r="AB6" s="68"/>
+      <c r="AC6" s="68"/>
+      <c r="AD6" s="68"/>
+      <c r="AE6" s="68"/>
       <c r="AF6" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="31" t="s">
         <v>61</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="76"/>
-      <c r="J7" s="76"/>
-      <c r="K7" s="76"/>
-      <c r="L7" s="76" t="s">
+      <c r="C7" s="110"/>
+      <c r="D7" s="110"/>
+      <c r="E7" s="110"/>
+      <c r="F7" s="110"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
+      <c r="I7" s="110"/>
+      <c r="J7" s="110"/>
+      <c r="K7" s="110"/>
+      <c r="L7" s="110" t="s">
         <v>60</v>
       </c>
-      <c r="M7" s="76"/>
-      <c r="N7" s="76"/>
-      <c r="O7" s="76"/>
-      <c r="P7" s="76"/>
-      <c r="Q7" s="76"/>
-      <c r="R7" s="76"/>
-      <c r="S7" s="76"/>
-      <c r="T7" s="76"/>
-      <c r="U7" s="76"/>
-      <c r="V7" s="76"/>
-      <c r="W7" s="77" t="s">
+      <c r="M7" s="110"/>
+      <c r="N7" s="110"/>
+      <c r="O7" s="110"/>
+      <c r="P7" s="110"/>
+      <c r="Q7" s="110"/>
+      <c r="R7" s="110"/>
+      <c r="S7" s="110"/>
+      <c r="T7" s="110"/>
+      <c r="U7" s="110"/>
+      <c r="V7" s="110"/>
+      <c r="W7" s="111" t="s">
         <v>62</v>
       </c>
-      <c r="X7" s="77"/>
-      <c r="Y7" s="77"/>
-      <c r="Z7" s="77"/>
-      <c r="AA7" s="77"/>
-      <c r="AB7" s="77"/>
-      <c r="AC7" s="77"/>
-      <c r="AD7" s="77"/>
-      <c r="AE7" s="76"/>
-      <c r="AF7" s="76"/>
-    </row>
-    <row r="8" spans="1:32" s="7" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A8" s="96" t="s">
+      <c r="X7" s="111"/>
+      <c r="Y7" s="111"/>
+      <c r="Z7" s="111"/>
+      <c r="AA7" s="111"/>
+      <c r="AB7" s="111"/>
+      <c r="AC7" s="111"/>
+      <c r="AD7" s="111"/>
+      <c r="AE7" s="110"/>
+      <c r="AF7" s="110"/>
+    </row>
+    <row r="8" spans="1:32" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A8" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="70"/>
-      <c r="D8" s="101" t="s">
+      <c r="C8" s="78"/>
+      <c r="D8" s="126" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="102"/>
-      <c r="F8" s="103" t="s">
+      <c r="E8" s="127"/>
+      <c r="F8" s="105" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="103"/>
-      <c r="H8" s="103" t="s">
+      <c r="G8" s="105"/>
+      <c r="H8" s="105" t="s">
         <v>71</v>
       </c>
-      <c r="I8" s="103"/>
-      <c r="J8" s="103" t="s">
+      <c r="I8" s="105"/>
+      <c r="J8" s="105" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="103"/>
-      <c r="L8" s="103" t="s">
+      <c r="K8" s="105"/>
+      <c r="L8" s="105" t="s">
         <v>72</v>
       </c>
-      <c r="M8" s="103"/>
-      <c r="N8" s="103" t="s">
+      <c r="M8" s="105"/>
+      <c r="N8" s="105" t="s">
         <v>73</v>
       </c>
-      <c r="O8" s="103"/>
-      <c r="P8" s="63" t="s">
+      <c r="O8" s="105"/>
+      <c r="P8" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="Q8" s="105" t="s">
+      <c r="Q8" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="R8" s="69" t="s">
+      <c r="R8" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="S8" s="70"/>
-      <c r="T8" s="103" t="s">
+      <c r="S8" s="78"/>
+      <c r="T8" s="105" t="s">
         <v>74</v>
       </c>
-      <c r="U8" s="103"/>
-      <c r="V8" s="103" t="s">
+      <c r="U8" s="105"/>
+      <c r="V8" s="105" t="s">
         <v>70</v>
       </c>
-      <c r="W8" s="52"/>
-      <c r="X8" s="52" t="s">
+      <c r="W8" s="73"/>
+      <c r="X8" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="Y8" s="52"/>
-      <c r="Z8" s="52" t="s">
+      <c r="Y8" s="73"/>
+      <c r="Z8" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="AA8" s="52"/>
-      <c r="AB8" s="52" t="s">
+      <c r="AA8" s="73"/>
+      <c r="AB8" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AC8" s="52"/>
-      <c r="AD8" s="52" t="s">
+      <c r="AC8" s="73"/>
+      <c r="AD8" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="AE8" s="103"/>
-      <c r="AF8" s="96" t="s">
+      <c r="AE8" s="105"/>
+      <c r="AF8" s="86" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="96"/>
-      <c r="B9" s="97"/>
-      <c r="C9" s="98"/>
+    <row r="9" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="86"/>
+      <c r="B9" s="100"/>
+      <c r="C9" s="101"/>
       <c r="D9" s="11" t="s">
         <v>10</v>
       </c>
@@ -2456,10 +2453,10 @@
       <c r="O9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="P9" s="104"/>
-      <c r="Q9" s="105"/>
-      <c r="R9" s="97"/>
-      <c r="S9" s="98"/>
+      <c r="P9" s="102"/>
+      <c r="Q9" s="106"/>
+      <c r="R9" s="100"/>
+      <c r="S9" s="101"/>
       <c r="T9" s="12" t="s">
         <v>10</v>
       </c>
@@ -2496,16 +2493,16 @@
       <c r="AE9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="AF9" s="100"/>
-    </row>
-    <row r="10" spans="1:32" s="7" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="78" t="s">
+      <c r="AF9" s="99"/>
+    </row>
+    <row r="10" spans="1:32" s="7" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="81" t="s">
+      <c r="B10" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="82"/>
+      <c r="C10" s="116"/>
       <c r="D10" s="43"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14"/>
@@ -2519,45 +2516,45 @@
       <c r="N10" s="14"/>
       <c r="O10" s="14"/>
       <c r="P10" s="15"/>
-      <c r="Q10" s="83" t="s">
+      <c r="Q10" s="117" t="s">
         <v>14</v>
       </c>
-      <c r="R10" s="86" t="s">
+      <c r="R10" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="S10" s="87"/>
+      <c r="S10" s="94"/>
       <c r="T10" s="16"/>
       <c r="U10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V10" s="16"/>
       <c r="W10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="X10" s="16"/>
       <c r="Y10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Z10" s="16"/>
       <c r="AA10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AB10" s="17"/>
       <c r="AC10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD10" s="17"/>
       <c r="AE10" s="29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AF10" s="17"/>
     </row>
-    <row r="11" spans="1:32" s="7" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="79"/>
-      <c r="B11" s="88" t="s">
+    <row r="11" spans="1:32" s="7" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="113"/>
+      <c r="B11" s="120" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="89"/>
+      <c r="C11" s="121"/>
       <c r="D11" s="43"/>
       <c r="E11" s="13"/>
       <c r="F11" s="14"/>
@@ -2571,43 +2568,43 @@
       <c r="N11" s="14"/>
       <c r="O11" s="14"/>
       <c r="P11" s="18"/>
-      <c r="Q11" s="84"/>
-      <c r="R11" s="90" t="s">
+      <c r="Q11" s="118"/>
+      <c r="R11" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="S11" s="91"/>
+      <c r="S11" s="72"/>
       <c r="T11" s="19"/>
       <c r="U11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V11" s="19"/>
       <c r="W11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="X11" s="19"/>
       <c r="Y11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Z11" s="19"/>
       <c r="AA11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AB11" s="14"/>
       <c r="AC11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD11" s="14"/>
       <c r="AE11" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AF11" s="14"/>
     </row>
-    <row r="12" spans="1:32" s="7" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="80"/>
-      <c r="B12" s="92" t="s">
+    <row r="12" spans="1:32" s="7" customFormat="1" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="114"/>
+      <c r="B12" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="93"/>
+      <c r="C12" s="122"/>
       <c r="D12" s="33"/>
       <c r="E12" s="20"/>
       <c r="F12" s="14"/>
@@ -2621,145 +2618,145 @@
       <c r="N12" s="14"/>
       <c r="O12" s="14"/>
       <c r="P12" s="21"/>
-      <c r="Q12" s="85"/>
-      <c r="R12" s="94" t="s">
+      <c r="Q12" s="119"/>
+      <c r="R12" s="123" t="s">
         <v>19</v>
       </c>
-      <c r="S12" s="95"/>
+      <c r="S12" s="124"/>
       <c r="T12" s="22"/>
       <c r="U12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V12" s="22"/>
       <c r="W12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="X12" s="22"/>
       <c r="Y12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Z12" s="22"/>
       <c r="AA12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AB12" s="23"/>
       <c r="AC12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AD12" s="23"/>
       <c r="AE12" s="30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AF12" s="23"/>
     </row>
-    <row r="13" spans="1:32" s="7" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="106"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="65"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="65"/>
-      <c r="G13" s="65"/>
-      <c r="H13" s="65"/>
-      <c r="I13" s="65"/>
-      <c r="J13" s="65"/>
-      <c r="K13" s="65"/>
-      <c r="L13" s="65"/>
-      <c r="M13" s="65"/>
-      <c r="N13" s="65"/>
-      <c r="O13" s="65"/>
-      <c r="P13" s="65"/>
-      <c r="Q13" s="65"/>
-      <c r="R13" s="65"/>
-      <c r="S13" s="65"/>
-      <c r="T13" s="65"/>
-      <c r="U13" s="65"/>
-      <c r="V13" s="65"/>
-      <c r="W13" s="65"/>
-      <c r="X13" s="65"/>
-      <c r="Y13" s="65"/>
-      <c r="Z13" s="65"/>
-      <c r="AA13" s="65"/>
-      <c r="AB13" s="65"/>
-      <c r="AC13" s="65"/>
-      <c r="AD13" s="65"/>
-      <c r="AE13" s="65"/>
-      <c r="AF13" s="107"/>
-    </row>
-    <row r="14" spans="1:32" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="108" t="s">
+    <row r="13" spans="1:32" s="7" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="83"/>
+      <c r="B13" s="84"/>
+      <c r="C13" s="84"/>
+      <c r="D13" s="84"/>
+      <c r="E13" s="84"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="84"/>
+      <c r="H13" s="84"/>
+      <c r="I13" s="84"/>
+      <c r="J13" s="84"/>
+      <c r="K13" s="84"/>
+      <c r="L13" s="84"/>
+      <c r="M13" s="84"/>
+      <c r="N13" s="84"/>
+      <c r="O13" s="84"/>
+      <c r="P13" s="84"/>
+      <c r="Q13" s="84"/>
+      <c r="R13" s="84"/>
+      <c r="S13" s="84"/>
+      <c r="T13" s="84"/>
+      <c r="U13" s="84"/>
+      <c r="V13" s="84"/>
+      <c r="W13" s="84"/>
+      <c r="X13" s="84"/>
+      <c r="Y13" s="84"/>
+      <c r="Z13" s="84"/>
+      <c r="AA13" s="84"/>
+      <c r="AB13" s="84"/>
+      <c r="AC13" s="84"/>
+      <c r="AD13" s="84"/>
+      <c r="AE13" s="84"/>
+      <c r="AF13" s="98"/>
+    </row>
+    <row r="14" spans="1:32" s="7" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="67" t="s">
+      <c r="B14" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="68"/>
-      <c r="D14" s="52" t="s">
+      <c r="C14" s="76"/>
+      <c r="D14" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52" t="s">
+      <c r="E14" s="73"/>
+      <c r="F14" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52" t="s">
+      <c r="G14" s="73"/>
+      <c r="H14" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="I14" s="52"/>
-      <c r="J14" s="52" t="s">
+      <c r="I14" s="73"/>
+      <c r="J14" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="K14" s="52"/>
-      <c r="L14" s="52" t="s">
+      <c r="K14" s="73"/>
+      <c r="L14" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="M14" s="52"/>
-      <c r="N14" s="52" t="s">
+      <c r="M14" s="73"/>
+      <c r="N14" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="O14" s="52"/>
-      <c r="P14" s="62" t="s">
+      <c r="O14" s="73"/>
+      <c r="P14" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="Q14" s="109" t="s">
+      <c r="Q14" s="103" t="s">
         <v>7</v>
       </c>
-      <c r="R14" s="67" t="s">
+      <c r="R14" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="S14" s="68"/>
-      <c r="T14" s="52" t="s">
+      <c r="S14" s="76"/>
+      <c r="T14" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="U14" s="52"/>
-      <c r="V14" s="52" t="s">
+      <c r="U14" s="73"/>
+      <c r="V14" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="W14" s="52"/>
-      <c r="X14" s="52" t="s">
+      <c r="W14" s="73"/>
+      <c r="X14" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="Y14" s="52"/>
-      <c r="Z14" s="52" t="s">
+      <c r="Y14" s="73"/>
+      <c r="Z14" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="AA14" s="52"/>
-      <c r="AB14" s="52" t="s">
+      <c r="AA14" s="73"/>
+      <c r="AB14" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AC14" s="52"/>
-      <c r="AD14" s="52" t="s">
+      <c r="AC14" s="73"/>
+      <c r="AD14" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="AE14" s="52"/>
-      <c r="AF14" s="108" t="s">
+      <c r="AE14" s="73"/>
+      <c r="AF14" s="85" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="100"/>
-      <c r="B15" s="97"/>
-      <c r="C15" s="98"/>
+    <row r="15" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="99"/>
+      <c r="B15" s="100"/>
+      <c r="C15" s="101"/>
       <c r="D15" s="12" t="s">
         <v>10</v>
       </c>
@@ -2796,10 +2793,10 @@
       <c r="O15" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="P15" s="104"/>
-      <c r="Q15" s="110"/>
-      <c r="R15" s="97"/>
-      <c r="S15" s="98"/>
+      <c r="P15" s="102"/>
+      <c r="Q15" s="104"/>
+      <c r="R15" s="100"/>
+      <c r="S15" s="101"/>
       <c r="T15" s="24" t="s">
         <v>10</v>
       </c>
@@ -2836,16 +2833,16 @@
       <c r="AE15" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="AF15" s="100"/>
-    </row>
-    <row r="16" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="113" t="s">
+      <c r="AF15" s="99"/>
+    </row>
+    <row r="16" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="119" t="s">
+      <c r="B16" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="120"/>
+      <c r="C16" s="97"/>
       <c r="D16" s="43"/>
       <c r="E16" s="13"/>
       <c r="F16" s="14"/>
@@ -2859,13 +2856,13 @@
       <c r="N16" s="14"/>
       <c r="O16" s="14"/>
       <c r="P16" s="15"/>
-      <c r="Q16" s="116" t="s">
+      <c r="Q16" s="90" t="s">
         <v>22</v>
       </c>
-      <c r="R16" s="86" t="s">
+      <c r="R16" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="S16" s="87"/>
+      <c r="S16" s="94"/>
       <c r="T16" s="13"/>
       <c r="U16" s="13"/>
       <c r="V16" s="14"/>
@@ -2880,12 +2877,12 @@
       <c r="AE16" s="14"/>
       <c r="AF16" s="17"/>
     </row>
-    <row r="17" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="114"/>
-      <c r="B17" s="74" t="s">
+    <row r="17" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="88"/>
+      <c r="B17" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="75"/>
+      <c r="C17" s="95"/>
       <c r="D17" s="43"/>
       <c r="E17" s="13"/>
       <c r="F17" s="14"/>
@@ -2899,11 +2896,11 @@
       <c r="N17" s="14"/>
       <c r="O17" s="14"/>
       <c r="P17" s="18"/>
-      <c r="Q17" s="117"/>
-      <c r="R17" s="90" t="s">
+      <c r="Q17" s="91"/>
+      <c r="R17" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="S17" s="91"/>
+      <c r="S17" s="72"/>
       <c r="T17" s="13"/>
       <c r="U17" s="13"/>
       <c r="V17" s="14"/>
@@ -2918,12 +2915,12 @@
       <c r="AE17" s="14"/>
       <c r="AF17" s="14"/>
     </row>
-    <row r="18" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="114"/>
-      <c r="B18" s="74" t="s">
+    <row r="18" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="88"/>
+      <c r="B18" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="74"/>
+      <c r="C18" s="68"/>
       <c r="D18" s="33"/>
       <c r="E18" s="20"/>
       <c r="F18" s="14"/>
@@ -2937,11 +2934,11 @@
       <c r="N18" s="14"/>
       <c r="O18" s="14"/>
       <c r="P18" s="18"/>
-      <c r="Q18" s="117"/>
-      <c r="R18" s="90" t="s">
+      <c r="Q18" s="91"/>
+      <c r="R18" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="S18" s="91"/>
+      <c r="S18" s="72"/>
       <c r="T18" s="20"/>
       <c r="U18" s="20"/>
       <c r="V18" s="14"/>
@@ -2956,12 +2953,12 @@
       <c r="AE18" s="14"/>
       <c r="AF18" s="14"/>
     </row>
-    <row r="19" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="114"/>
-      <c r="B19" s="74" t="s">
+    <row r="19" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="88"/>
+      <c r="B19" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="74"/>
+      <c r="C19" s="68"/>
       <c r="D19" s="33"/>
       <c r="E19" s="20"/>
       <c r="F19" s="14"/>
@@ -2975,11 +2972,11 @@
       <c r="N19" s="14"/>
       <c r="O19" s="14"/>
       <c r="P19" s="18"/>
-      <c r="Q19" s="117"/>
-      <c r="R19" s="90" t="s">
+      <c r="Q19" s="91"/>
+      <c r="R19" s="71" t="s">
         <v>29</v>
       </c>
-      <c r="S19" s="91"/>
+      <c r="S19" s="72"/>
       <c r="T19" s="20"/>
       <c r="U19" s="20"/>
       <c r="V19" s="14"/>
@@ -2994,12 +2991,12 @@
       <c r="AE19" s="14"/>
       <c r="AF19" s="14"/>
     </row>
-    <row r="20" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="114"/>
-      <c r="B20" s="74" t="s">
+    <row r="20" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="88"/>
+      <c r="B20" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="74"/>
+      <c r="C20" s="68"/>
       <c r="D20" s="33"/>
       <c r="E20" s="20"/>
       <c r="F20" s="14"/>
@@ -3013,11 +3010,11 @@
       <c r="N20" s="14"/>
       <c r="O20" s="14"/>
       <c r="P20" s="18"/>
-      <c r="Q20" s="117"/>
-      <c r="R20" s="90" t="s">
+      <c r="Q20" s="91"/>
+      <c r="R20" s="71" t="s">
         <v>31</v>
       </c>
-      <c r="S20" s="91"/>
+      <c r="S20" s="72"/>
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
       <c r="V20" s="14"/>
@@ -3032,12 +3029,12 @@
       <c r="AE20" s="14"/>
       <c r="AF20" s="14"/>
     </row>
-    <row r="21" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="114"/>
-      <c r="B21" s="74" t="s">
+    <row r="21" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="88"/>
+      <c r="B21" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="74"/>
+      <c r="C21" s="68"/>
       <c r="D21" s="33"/>
       <c r="E21" s="20"/>
       <c r="F21" s="14"/>
@@ -3051,11 +3048,11 @@
       <c r="N21" s="14"/>
       <c r="O21" s="14"/>
       <c r="P21" s="18"/>
-      <c r="Q21" s="117"/>
-      <c r="R21" s="90" t="s">
+      <c r="Q21" s="91"/>
+      <c r="R21" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="S21" s="91"/>
+      <c r="S21" s="72"/>
       <c r="T21" s="20"/>
       <c r="U21" s="20"/>
       <c r="V21" s="14"/>
@@ -3070,12 +3067,12 @@
       <c r="AE21" s="14"/>
       <c r="AF21" s="14"/>
     </row>
-    <row r="22" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="114"/>
-      <c r="B22" s="74" t="s">
+    <row r="22" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="88"/>
+      <c r="B22" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="74"/>
+      <c r="C22" s="68"/>
       <c r="D22" s="33"/>
       <c r="E22" s="20"/>
       <c r="F22" s="14"/>
@@ -3089,11 +3086,11 @@
       <c r="N22" s="14"/>
       <c r="O22" s="14"/>
       <c r="P22" s="18"/>
-      <c r="Q22" s="117"/>
-      <c r="R22" s="90" t="s">
+      <c r="Q22" s="91"/>
+      <c r="R22" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="S22" s="91"/>
+      <c r="S22" s="72"/>
       <c r="T22" s="20"/>
       <c r="U22" s="20"/>
       <c r="V22" s="14"/>
@@ -3108,12 +3105,12 @@
       <c r="AE22" s="14"/>
       <c r="AF22" s="14"/>
     </row>
-    <row r="23" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="114"/>
-      <c r="B23" s="74" t="s">
+    <row r="23" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="88"/>
+      <c r="B23" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="74"/>
+      <c r="C23" s="68"/>
       <c r="D23" s="33"/>
       <c r="E23" s="20"/>
       <c r="F23" s="14"/>
@@ -3127,11 +3124,11 @@
       <c r="N23" s="14"/>
       <c r="O23" s="14"/>
       <c r="P23" s="18"/>
-      <c r="Q23" s="117"/>
-      <c r="R23" s="90" t="s">
+      <c r="Q23" s="91"/>
+      <c r="R23" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="S23" s="91"/>
+      <c r="S23" s="72"/>
       <c r="T23" s="20"/>
       <c r="U23" s="20"/>
       <c r="V23" s="14"/>
@@ -3146,12 +3143,12 @@
       <c r="AE23" s="14"/>
       <c r="AF23" s="14"/>
     </row>
-    <row r="24" spans="1:32" s="7" customFormat="1" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="114"/>
-      <c r="B24" s="74" t="s">
+    <row r="24" spans="1:32" s="7" customFormat="1" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="88"/>
+      <c r="B24" s="68" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="74"/>
+      <c r="C24" s="68"/>
       <c r="D24" s="33"/>
       <c r="E24" s="20"/>
       <c r="F24" s="14"/>
@@ -3165,11 +3162,11 @@
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
       <c r="P24" s="18"/>
-      <c r="Q24" s="118"/>
-      <c r="R24" s="138" t="s">
+      <c r="Q24" s="92"/>
+      <c r="R24" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="S24" s="139"/>
+      <c r="S24" s="70"/>
       <c r="T24" s="20"/>
       <c r="U24" s="20"/>
       <c r="V24" s="14"/>
@@ -3184,12 +3181,12 @@
       <c r="AE24" s="14"/>
       <c r="AF24" s="23"/>
     </row>
-    <row r="25" spans="1:32" s="7" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A25" s="114"/>
-      <c r="B25" s="74" t="s">
+    <row r="25" spans="1:32" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A25" s="88"/>
+      <c r="B25" s="68" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="74"/>
+      <c r="C25" s="68"/>
       <c r="D25" s="33"/>
       <c r="E25" s="20"/>
       <c r="F25" s="14"/>
@@ -3203,29 +3200,29 @@
       <c r="N25" s="14"/>
       <c r="O25" s="14"/>
       <c r="P25" s="18"/>
-      <c r="Q25" s="111"/>
-      <c r="R25" s="111"/>
-      <c r="S25" s="111"/>
-      <c r="T25" s="111"/>
-      <c r="U25" s="111"/>
-      <c r="V25" s="111"/>
-      <c r="W25" s="111"/>
-      <c r="X25" s="111"/>
-      <c r="Y25" s="111"/>
-      <c r="Z25" s="111"/>
-      <c r="AA25" s="111"/>
-      <c r="AB25" s="111"/>
-      <c r="AC25" s="111"/>
-      <c r="AD25" s="111"/>
-      <c r="AE25" s="111"/>
-      <c r="AF25" s="112"/>
-    </row>
-    <row r="26" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="115"/>
-      <c r="B26" s="92" t="s">
+      <c r="Q25" s="81"/>
+      <c r="R25" s="81"/>
+      <c r="S25" s="81"/>
+      <c r="T25" s="81"/>
+      <c r="U25" s="81"/>
+      <c r="V25" s="81"/>
+      <c r="W25" s="81"/>
+      <c r="X25" s="81"/>
+      <c r="Y25" s="81"/>
+      <c r="Z25" s="81"/>
+      <c r="AA25" s="81"/>
+      <c r="AB25" s="81"/>
+      <c r="AC25" s="81"/>
+      <c r="AD25" s="81"/>
+      <c r="AE25" s="81"/>
+      <c r="AF25" s="82"/>
+    </row>
+    <row r="26" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="89"/>
+      <c r="B26" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="92"/>
+      <c r="C26" s="74"/>
       <c r="D26" s="33"/>
       <c r="E26" s="20"/>
       <c r="F26" s="14"/>
@@ -3239,131 +3236,131 @@
       <c r="N26" s="14"/>
       <c r="O26" s="14"/>
       <c r="P26" s="21"/>
-      <c r="Q26" s="111"/>
-      <c r="R26" s="111"/>
-      <c r="S26" s="111"/>
-      <c r="T26" s="111"/>
-      <c r="U26" s="111"/>
-      <c r="V26" s="111"/>
-      <c r="W26" s="111"/>
-      <c r="X26" s="111"/>
-      <c r="Y26" s="111"/>
-      <c r="Z26" s="111"/>
-      <c r="AA26" s="111"/>
-      <c r="AB26" s="111"/>
-      <c r="AC26" s="111"/>
-      <c r="AD26" s="111"/>
-      <c r="AE26" s="111"/>
-      <c r="AF26" s="112"/>
-    </row>
-    <row r="27" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="106"/>
-      <c r="B27" s="65"/>
-      <c r="C27" s="65"/>
-      <c r="D27" s="65"/>
-      <c r="E27" s="65"/>
-      <c r="F27" s="65"/>
-      <c r="G27" s="65"/>
-      <c r="H27" s="65"/>
-      <c r="I27" s="65"/>
-      <c r="J27" s="65"/>
-      <c r="K27" s="65"/>
-      <c r="L27" s="65"/>
-      <c r="M27" s="65"/>
-      <c r="N27" s="65"/>
-      <c r="O27" s="65"/>
-      <c r="P27" s="65"/>
-      <c r="Q27" s="111"/>
-      <c r="R27" s="111"/>
-      <c r="S27" s="111"/>
-      <c r="T27" s="111"/>
-      <c r="U27" s="111"/>
-      <c r="V27" s="111"/>
-      <c r="W27" s="111"/>
-      <c r="X27" s="111"/>
-      <c r="Y27" s="111"/>
-      <c r="Z27" s="111"/>
-      <c r="AA27" s="111"/>
-      <c r="AB27" s="111"/>
-      <c r="AC27" s="111"/>
-      <c r="AD27" s="111"/>
-      <c r="AE27" s="111"/>
-      <c r="AF27" s="112"/>
-    </row>
-    <row r="28" spans="1:32" s="7" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A28" s="108" t="s">
+      <c r="Q26" s="81"/>
+      <c r="R26" s="81"/>
+      <c r="S26" s="81"/>
+      <c r="T26" s="81"/>
+      <c r="U26" s="81"/>
+      <c r="V26" s="81"/>
+      <c r="W26" s="81"/>
+      <c r="X26" s="81"/>
+      <c r="Y26" s="81"/>
+      <c r="Z26" s="81"/>
+      <c r="AA26" s="81"/>
+      <c r="AB26" s="81"/>
+      <c r="AC26" s="81"/>
+      <c r="AD26" s="81"/>
+      <c r="AE26" s="81"/>
+      <c r="AF26" s="82"/>
+    </row>
+    <row r="27" spans="1:32" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="83"/>
+      <c r="B27" s="84"/>
+      <c r="C27" s="84"/>
+      <c r="D27" s="84"/>
+      <c r="E27" s="84"/>
+      <c r="F27" s="84"/>
+      <c r="G27" s="84"/>
+      <c r="H27" s="84"/>
+      <c r="I27" s="84"/>
+      <c r="J27" s="84"/>
+      <c r="K27" s="84"/>
+      <c r="L27" s="84"/>
+      <c r="M27" s="84"/>
+      <c r="N27" s="84"/>
+      <c r="O27" s="84"/>
+      <c r="P27" s="84"/>
+      <c r="Q27" s="81"/>
+      <c r="R27" s="81"/>
+      <c r="S27" s="81"/>
+      <c r="T27" s="81"/>
+      <c r="U27" s="81"/>
+      <c r="V27" s="81"/>
+      <c r="W27" s="81"/>
+      <c r="X27" s="81"/>
+      <c r="Y27" s="81"/>
+      <c r="Z27" s="81"/>
+      <c r="AA27" s="81"/>
+      <c r="AB27" s="81"/>
+      <c r="AC27" s="81"/>
+      <c r="AD27" s="81"/>
+      <c r="AE27" s="81"/>
+      <c r="AF27" s="82"/>
+    </row>
+    <row r="28" spans="1:32" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A28" s="85" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="67" t="s">
+      <c r="B28" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="68"/>
-      <c r="D28" s="52" t="s">
+      <c r="C28" s="76"/>
+      <c r="D28" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52" t="s">
+      <c r="E28" s="73"/>
+      <c r="F28" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52" t="s">
+      <c r="G28" s="73"/>
+      <c r="H28" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="I28" s="52"/>
-      <c r="J28" s="52" t="s">
+      <c r="I28" s="73"/>
+      <c r="J28" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="K28" s="52"/>
-      <c r="L28" s="52" t="s">
+      <c r="K28" s="73"/>
+      <c r="L28" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="M28" s="52"/>
-      <c r="N28" s="52" t="s">
+      <c r="M28" s="73"/>
+      <c r="N28" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="O28" s="52"/>
-      <c r="P28" s="62" t="s">
+      <c r="O28" s="73"/>
+      <c r="P28" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="Q28" s="136" t="s">
+      <c r="Q28" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="R28" s="133" t="s">
+      <c r="R28" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="S28" s="133"/>
-      <c r="T28" s="52" t="s">
+      <c r="S28" s="62"/>
+      <c r="T28" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="U28" s="52"/>
-      <c r="V28" s="52" t="s">
+      <c r="U28" s="73"/>
+      <c r="V28" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="W28" s="52"/>
-      <c r="X28" s="52" t="s">
+      <c r="W28" s="73"/>
+      <c r="X28" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="Y28" s="52"/>
-      <c r="Z28" s="52" t="s">
+      <c r="Y28" s="73"/>
+      <c r="Z28" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="AA28" s="52"/>
-      <c r="AB28" s="52" t="s">
+      <c r="AA28" s="73"/>
+      <c r="AB28" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AC28" s="52"/>
-      <c r="AD28" s="52" t="s">
+      <c r="AC28" s="73"/>
+      <c r="AD28" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="AE28" s="52"/>
-      <c r="AF28" s="133" t="s">
+      <c r="AE28" s="73"/>
+      <c r="AF28" s="62" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:32" s="7" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A29" s="96"/>
-      <c r="B29" s="69"/>
-      <c r="C29" s="70"/>
+    <row r="29" spans="1:32" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A29" s="86"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="78"/>
       <c r="D29" s="11" t="s">
         <v>10</v>
       </c>
@@ -3400,10 +3397,10 @@
       <c r="O29" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="P29" s="63"/>
-      <c r="Q29" s="137"/>
-      <c r="R29" s="134"/>
-      <c r="S29" s="134"/>
+      <c r="P29" s="80"/>
+      <c r="Q29" s="67"/>
+      <c r="R29" s="63"/>
+      <c r="S29" s="63"/>
       <c r="T29" s="9" t="s">
         <v>10</v>
       </c>
@@ -3440,16 +3437,16 @@
       <c r="AE29" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="AF29" s="134"/>
-    </row>
-    <row r="30" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="56" t="s">
+      <c r="AF29" s="63"/>
+    </row>
+    <row r="30" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="129" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="57" t="s">
+      <c r="B30" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="57"/>
+      <c r="C30" s="65"/>
       <c r="D30" s="43"/>
       <c r="E30" s="13"/>
       <c r="F30" s="14"/>
@@ -3463,13 +3460,13 @@
       <c r="N30" s="14"/>
       <c r="O30" s="14"/>
       <c r="P30" s="14"/>
-      <c r="Q30" s="135" t="s">
+      <c r="Q30" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="R30" s="57" t="s">
+      <c r="R30" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="S30" s="57"/>
+      <c r="S30" s="65"/>
       <c r="T30" s="13"/>
       <c r="U30" s="13"/>
       <c r="V30" s="14"/>
@@ -3484,12 +3481,12 @@
       <c r="AE30" s="14"/>
       <c r="AF30" s="14"/>
     </row>
-    <row r="31" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="56"/>
-      <c r="B31" s="57" t="s">
+    <row r="31" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="129"/>
+      <c r="B31" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="57"/>
+      <c r="C31" s="65"/>
       <c r="D31" s="43"/>
       <c r="E31" s="13"/>
       <c r="F31" s="14"/>
@@ -3503,11 +3500,11 @@
       <c r="N31" s="14"/>
       <c r="O31" s="14"/>
       <c r="P31" s="14"/>
-      <c r="Q31" s="135"/>
-      <c r="R31" s="57" t="s">
+      <c r="Q31" s="64"/>
+      <c r="R31" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="S31" s="57"/>
+      <c r="S31" s="65"/>
       <c r="T31" s="13"/>
       <c r="U31" s="13"/>
       <c r="V31" s="14"/>
@@ -3522,12 +3519,12 @@
       <c r="AE31" s="14"/>
       <c r="AF31" s="14"/>
     </row>
-    <row r="32" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="56"/>
-      <c r="B32" s="57" t="s">
+    <row r="32" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="129"/>
+      <c r="B32" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="C32" s="57"/>
+      <c r="C32" s="65"/>
       <c r="D32" s="44"/>
       <c r="E32" s="25"/>
       <c r="F32" s="14"/>
@@ -3541,11 +3538,11 @@
       <c r="N32" s="14"/>
       <c r="O32" s="14"/>
       <c r="P32" s="14"/>
-      <c r="Q32" s="135"/>
-      <c r="R32" s="57" t="s">
+      <c r="Q32" s="64"/>
+      <c r="R32" s="65" t="s">
         <v>57</v>
       </c>
-      <c r="S32" s="57"/>
+      <c r="S32" s="65"/>
       <c r="T32" s="25"/>
       <c r="U32" s="25"/>
       <c r="V32" s="25"/>
@@ -3560,12 +3557,12 @@
       <c r="AE32" s="14"/>
       <c r="AF32" s="14"/>
     </row>
-    <row r="33" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="56"/>
-      <c r="B33" s="57" t="s">
+    <row r="33" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="129"/>
+      <c r="B33" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="57"/>
+      <c r="C33" s="65"/>
       <c r="D33" s="44"/>
       <c r="E33" s="25"/>
       <c r="F33" s="14"/>
@@ -3579,11 +3576,11 @@
       <c r="N33" s="14"/>
       <c r="O33" s="14"/>
       <c r="P33" s="14"/>
-      <c r="Q33" s="135"/>
-      <c r="R33" s="57" t="s">
+      <c r="Q33" s="64"/>
+      <c r="R33" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="S33" s="57"/>
+      <c r="S33" s="65"/>
       <c r="T33" s="25"/>
       <c r="U33" s="25"/>
       <c r="V33" s="25"/>
@@ -3598,12 +3595,12 @@
       <c r="AE33" s="14"/>
       <c r="AF33" s="14"/>
     </row>
-    <row r="34" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="56"/>
-      <c r="B34" s="57" t="s">
+    <row r="34" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="129"/>
+      <c r="B34" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="57"/>
+      <c r="C34" s="65"/>
       <c r="D34" s="44"/>
       <c r="E34" s="25"/>
       <c r="F34" s="14"/>
@@ -3617,11 +3614,11 @@
       <c r="N34" s="14"/>
       <c r="O34" s="14"/>
       <c r="P34" s="14"/>
-      <c r="Q34" s="135"/>
-      <c r="R34" s="57" t="s">
+      <c r="Q34" s="64"/>
+      <c r="R34" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="S34" s="57"/>
+      <c r="S34" s="65"/>
       <c r="T34" s="25"/>
       <c r="U34" s="25"/>
       <c r="V34" s="25"/>
@@ -3636,12 +3633,12 @@
       <c r="AE34" s="14"/>
       <c r="AF34" s="14"/>
     </row>
-    <row r="35" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="56"/>
-      <c r="B35" s="57" t="s">
+    <row r="35" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="129"/>
+      <c r="B35" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="57"/>
+      <c r="C35" s="65"/>
       <c r="D35" s="44"/>
       <c r="E35" s="25"/>
       <c r="F35" s="14"/>
@@ -3672,12 +3669,12 @@
       <c r="AE35"/>
       <c r="AF35"/>
     </row>
-    <row r="36" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="56"/>
-      <c r="B36" s="57" t="s">
+    <row r="36" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="129"/>
+      <c r="B36" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="57"/>
+      <c r="C36" s="65"/>
       <c r="D36" s="44"/>
       <c r="E36" s="25"/>
       <c r="F36" s="14"/>
@@ -3708,23 +3705,23 @@
       <c r="AE36"/>
       <c r="AF36"/>
     </row>
-    <row r="37" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="65"/>
-      <c r="B37" s="65"/>
-      <c r="C37" s="65"/>
-      <c r="D37" s="65"/>
-      <c r="E37" s="65"/>
-      <c r="F37" s="65"/>
-      <c r="G37" s="65"/>
-      <c r="H37" s="65"/>
-      <c r="I37" s="65"/>
-      <c r="J37" s="65"/>
-      <c r="K37" s="65"/>
-      <c r="L37" s="65"/>
-      <c r="M37" s="65"/>
-      <c r="N37" s="65"/>
-      <c r="O37" s="65"/>
-      <c r="P37" s="65"/>
+    <row r="37" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="84"/>
+      <c r="B37" s="84"/>
+      <c r="C37" s="84"/>
+      <c r="D37" s="84"/>
+      <c r="E37" s="84"/>
+      <c r="F37" s="84"/>
+      <c r="G37" s="84"/>
+      <c r="H37" s="84"/>
+      <c r="I37" s="84"/>
+      <c r="J37" s="84"/>
+      <c r="K37" s="84"/>
+      <c r="L37" s="84"/>
+      <c r="M37" s="84"/>
+      <c r="N37" s="84"/>
+      <c r="O37" s="84"/>
+      <c r="P37" s="84"/>
       <c r="Q37"/>
       <c r="R37"/>
       <c r="S37"/>
@@ -3742,23 +3739,23 @@
       <c r="AE37"/>
       <c r="AF37"/>
     </row>
-    <row r="38" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="65"/>
-      <c r="B38" s="65"/>
-      <c r="C38" s="65"/>
-      <c r="D38" s="65"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="65"/>
-      <c r="I38" s="65"/>
-      <c r="J38" s="65"/>
-      <c r="K38" s="65"/>
-      <c r="L38" s="65"/>
-      <c r="M38" s="65"/>
-      <c r="N38" s="65"/>
-      <c r="O38" s="65"/>
-      <c r="P38" s="65"/>
+    <row r="38" spans="1:32" s="7" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="84"/>
+      <c r="B38" s="84"/>
+      <c r="C38" s="84"/>
+      <c r="D38" s="84"/>
+      <c r="E38" s="84"/>
+      <c r="F38" s="84"/>
+      <c r="G38" s="84"/>
+      <c r="H38" s="84"/>
+      <c r="I38" s="84"/>
+      <c r="J38" s="84"/>
+      <c r="K38" s="84"/>
+      <c r="L38" s="84"/>
+      <c r="M38" s="84"/>
+      <c r="N38" s="84"/>
+      <c r="O38" s="84"/>
+      <c r="P38" s="84"/>
       <c r="Q38"/>
       <c r="R38"/>
       <c r="S38"/>
@@ -3776,96 +3773,96 @@
       <c r="AE38"/>
       <c r="AF38"/>
     </row>
-    <row r="39" spans="1:32" s="7" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A39" s="65"/>
-      <c r="B39" s="65"/>
-      <c r="C39" s="65"/>
-      <c r="D39" s="65"/>
-      <c r="E39" s="65"/>
-      <c r="F39" s="65"/>
-      <c r="G39" s="65"/>
-      <c r="H39" s="65"/>
-      <c r="I39" s="65"/>
-      <c r="J39" s="65"/>
-      <c r="K39" s="65"/>
-      <c r="L39" s="65"/>
-      <c r="M39" s="65"/>
-      <c r="N39" s="65"/>
-      <c r="O39" s="65"/>
-      <c r="P39" s="65"/>
-      <c r="Q39" s="52" t="s">
+    <row r="39" spans="1:32" s="7" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A39" s="84"/>
+      <c r="B39" s="84"/>
+      <c r="C39" s="84"/>
+      <c r="D39" s="84"/>
+      <c r="E39" s="84"/>
+      <c r="F39" s="84"/>
+      <c r="G39" s="84"/>
+      <c r="H39" s="84"/>
+      <c r="I39" s="84"/>
+      <c r="J39" s="84"/>
+      <c r="K39" s="84"/>
+      <c r="L39" s="84"/>
+      <c r="M39" s="84"/>
+      <c r="N39" s="84"/>
+      <c r="O39" s="84"/>
+      <c r="P39" s="84"/>
+      <c r="Q39" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="R39" s="67" t="s">
+      <c r="R39" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="S39" s="68"/>
-      <c r="T39" s="52" t="s">
+      <c r="S39" s="76"/>
+      <c r="T39" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="U39" s="52"/>
-      <c r="V39" s="52" t="s">
+      <c r="U39" s="73"/>
+      <c r="V39" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="W39" s="52"/>
-      <c r="X39" s="52" t="s">
+      <c r="W39" s="73"/>
+      <c r="X39" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="Y39" s="52"/>
-      <c r="Z39" s="52" t="s">
+      <c r="Y39" s="73"/>
+      <c r="Z39" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="AA39" s="52"/>
-      <c r="AB39" s="52" t="s">
+      <c r="AA39" s="73"/>
+      <c r="AB39" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="AC39" s="52"/>
-      <c r="AD39" s="52" t="s">
+      <c r="AC39" s="73"/>
+      <c r="AD39" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="AE39" s="52"/>
-      <c r="AF39" s="62" t="s">
+      <c r="AE39" s="73"/>
+      <c r="AF39" s="79" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:32" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="52" t="s">
+    <row r="40" spans="1:32" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="B40" s="52" t="s">
+      <c r="B40" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="52"/>
-      <c r="D40" s="52" t="s">
+      <c r="C40" s="73"/>
+      <c r="D40" s="73" t="s">
         <v>74</v>
       </c>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52" t="s">
+      <c r="E40" s="73"/>
+      <c r="F40" s="73" t="s">
         <v>70</v>
       </c>
-      <c r="G40" s="52"/>
-      <c r="H40" s="52" t="s">
+      <c r="G40" s="73"/>
+      <c r="H40" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="I40" s="52"/>
-      <c r="J40" s="52" t="s">
+      <c r="I40" s="73"/>
+      <c r="J40" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="K40" s="52"/>
-      <c r="L40" s="52" t="s">
+      <c r="K40" s="73"/>
+      <c r="L40" s="73" t="s">
         <v>72</v>
       </c>
-      <c r="M40" s="52"/>
-      <c r="N40" s="52" t="s">
+      <c r="M40" s="73"/>
+      <c r="N40" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="O40" s="52"/>
-      <c r="P40" s="66" t="s">
+      <c r="O40" s="73"/>
+      <c r="P40" s="130" t="s">
         <v>9</v>
       </c>
-      <c r="Q40" s="52"/>
-      <c r="R40" s="69"/>
-      <c r="S40" s="70"/>
+      <c r="Q40" s="73"/>
+      <c r="R40" s="77"/>
+      <c r="S40" s="78"/>
       <c r="T40" s="9" t="s">
         <v>10</v>
       </c>
@@ -3902,12 +3899,12 @@
       <c r="AE40" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="AF40" s="63"/>
-    </row>
-    <row r="41" spans="1:32" s="7" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="52"/>
-      <c r="B41" s="52"/>
-      <c r="C41" s="52"/>
+      <c r="AF40" s="80"/>
+    </row>
+    <row r="41" spans="1:32" s="7" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="73"/>
+      <c r="B41" s="73"/>
+      <c r="C41" s="73"/>
       <c r="D41" s="12" t="s">
         <v>10</v>
       </c>
@@ -3944,14 +3941,14 @@
       <c r="O41" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="53" t="s">
-        <v>81</v>
-      </c>
-      <c r="R41" s="57" t="s">
+      <c r="P41" s="73"/>
+      <c r="Q41" s="131" t="s">
+        <v>80</v>
+      </c>
+      <c r="R41" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="S41" s="57"/>
+      <c r="S41" s="65"/>
       <c r="T41" s="13"/>
       <c r="U41" s="13"/>
       <c r="V41" s="14"/>
@@ -3966,14 +3963,14 @@
       <c r="AE41" s="14"/>
       <c r="AF41" s="14"/>
     </row>
-    <row r="42" spans="1:32" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="56" t="s">
+    <row r="42" spans="1:32" s="7" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="129" t="s">
         <v>50</v>
       </c>
-      <c r="B42" s="57" t="s">
+      <c r="B42" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="C42" s="57"/>
+      <c r="C42" s="65"/>
       <c r="D42" s="43"/>
       <c r="E42" s="13"/>
       <c r="F42" s="14"/>
@@ -3987,11 +3984,11 @@
       <c r="N42" s="14"/>
       <c r="O42" s="14"/>
       <c r="P42" s="14"/>
-      <c r="Q42" s="53"/>
-      <c r="R42" s="57" t="s">
+      <c r="Q42" s="131"/>
+      <c r="R42" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="S42" s="57"/>
+      <c r="S42" s="65"/>
       <c r="T42" s="13"/>
       <c r="U42" s="13"/>
       <c r="V42" s="14"/>
@@ -4006,12 +4003,12 @@
       <c r="AE42" s="14"/>
       <c r="AF42" s="14"/>
     </row>
-    <row r="43" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="56"/>
-      <c r="B43" s="57" t="s">
+    <row r="43" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="129"/>
+      <c r="B43" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="C43" s="57"/>
+      <c r="C43" s="65"/>
       <c r="D43" s="43"/>
       <c r="E43" s="13"/>
       <c r="F43" s="14"/>
@@ -4025,11 +4022,11 @@
       <c r="N43" s="14"/>
       <c r="O43" s="14"/>
       <c r="P43" s="14"/>
-      <c r="Q43" s="53"/>
-      <c r="R43" s="57" t="s">
+      <c r="Q43" s="131"/>
+      <c r="R43" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="S43" s="57"/>
+      <c r="S43" s="65"/>
       <c r="T43" s="25"/>
       <c r="U43" s="25"/>
       <c r="V43" s="14"/>
@@ -4044,12 +4041,12 @@
       <c r="AE43" s="14"/>
       <c r="AF43" s="14"/>
     </row>
-    <row r="44" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="56"/>
-      <c r="B44" s="57" t="s">
+    <row r="44" spans="1:32" s="7" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="129"/>
+      <c r="B44" s="65" t="s">
         <v>56</v>
       </c>
-      <c r="C44" s="57"/>
+      <c r="C44" s="65"/>
       <c r="D44" s="44"/>
       <c r="E44" s="25"/>
       <c r="F44" s="14"/>
@@ -4063,11 +4060,11 @@
       <c r="N44" s="14"/>
       <c r="O44" s="14"/>
       <c r="P44" s="14"/>
-      <c r="Q44" s="54"/>
-      <c r="R44" s="64" t="s">
+      <c r="Q44" s="132"/>
+      <c r="R44" s="128" t="s">
         <v>46</v>
       </c>
-      <c r="S44" s="64"/>
+      <c r="S44" s="128"/>
       <c r="T44" s="25"/>
       <c r="U44" s="25"/>
       <c r="V44" s="14"/>
@@ -4082,12 +4079,12 @@
       <c r="AE44" s="14"/>
       <c r="AF44" s="14"/>
     </row>
-    <row r="45" spans="1:32" s="7" customFormat="1" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="58" t="s">
-        <v>86</v>
-      </c>
-      <c r="B45" s="59"/>
-      <c r="C45" s="59"/>
+    <row r="45" spans="1:32" s="7" customFormat="1" ht="26.1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="134" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" s="135"/>
+      <c r="C45" s="135"/>
       <c r="D45" s="42"/>
       <c r="E45" s="37"/>
       <c r="F45" s="37"/>
@@ -4100,38 +4097,38 @@
       <c r="M45" s="37"/>
       <c r="N45" s="37"/>
       <c r="O45" s="37"/>
-      <c r="P45" s="55" t="s">
-        <v>87</v>
+      <c r="P45" s="133" t="s">
+        <v>86</v>
       </c>
       <c r="Q45" s="36"/>
-      <c r="R45" s="60"/>
-      <c r="S45" s="60"/>
-      <c r="T45" s="51" t="s">
+      <c r="R45" s="136"/>
+      <c r="S45" s="136"/>
+      <c r="T45" s="139" t="s">
         <v>74</v>
       </c>
-      <c r="U45" s="51"/>
-      <c r="V45" s="51" t="s">
+      <c r="U45" s="139"/>
+      <c r="V45" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="W45" s="51"/>
-      <c r="X45" s="51" t="s">
+      <c r="W45" s="139"/>
+      <c r="X45" s="139" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y45" s="139"/>
+      <c r="Z45" s="139" t="s">
         <v>84</v>
       </c>
-      <c r="Y45" s="51"/>
-      <c r="Z45" s="51" t="s">
-        <v>85</v>
-      </c>
-      <c r="AA45" s="51"/>
-      <c r="AB45" s="51" t="s">
+      <c r="AA45" s="139"/>
+      <c r="AB45" s="139" t="s">
         <v>72</v>
       </c>
-      <c r="AC45" s="51"/>
-      <c r="AD45" s="51" t="s">
+      <c r="AC45" s="139"/>
+      <c r="AD45" s="139" t="s">
         <v>73</v>
       </c>
-      <c r="AE45" s="51"/>
-    </row>
-    <row r="46" spans="1:32" s="7" customFormat="1" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AE45" s="139"/>
+    </row>
+    <row r="46" spans="1:32" s="7" customFormat="1" ht="26.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="48"/>
       <c r="B46" s="49"/>
       <c r="C46" s="49"/>
@@ -4147,27 +4144,27 @@
       <c r="M46" s="39"/>
       <c r="N46" s="39"/>
       <c r="O46" s="39"/>
-      <c r="P46" s="55"/>
+      <c r="P46" s="133"/>
       <c r="Q46" s="35"/>
-      <c r="R46" s="61" t="s">
-        <v>83</v>
-      </c>
-      <c r="S46" s="61"/>
-      <c r="T46" s="50"/>
-      <c r="U46" s="50"/>
-      <c r="V46" s="50"/>
-      <c r="W46" s="50"/>
-      <c r="X46" s="50"/>
-      <c r="Y46" s="50"/>
-      <c r="Z46" s="50"/>
-      <c r="AA46" s="50"/>
-      <c r="AB46" s="50"/>
-      <c r="AC46" s="50"/>
-      <c r="AD46" s="50"/>
-      <c r="AE46" s="50"/>
+      <c r="R46" s="137" t="s">
+        <v>82</v>
+      </c>
+      <c r="S46" s="137"/>
+      <c r="T46" s="138"/>
+      <c r="U46" s="138"/>
+      <c r="V46" s="138"/>
+      <c r="W46" s="138"/>
+      <c r="X46" s="138"/>
+      <c r="Y46" s="138"/>
+      <c r="Z46" s="138"/>
+      <c r="AA46" s="138"/>
+      <c r="AB46" s="138"/>
+      <c r="AC46" s="138"/>
+      <c r="AD46" s="138"/>
+      <c r="AE46" s="138"/>
       <c r="AF46"/>
     </row>
-    <row r="47" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="38"/>
       <c r="B47" s="39"/>
       <c r="C47" s="39"/>
@@ -4183,10 +4180,10 @@
       <c r="M47" s="39"/>
       <c r="N47" s="39"/>
       <c r="O47" s="39"/>
-      <c r="P47" s="55"/>
+      <c r="P47" s="133"/>
       <c r="Q47" s="27"/>
     </row>
-    <row r="48" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="40"/>
       <c r="B48" s="41"/>
       <c r="C48" s="41"/>
@@ -4202,16 +4199,16 @@
       <c r="M48" s="41"/>
       <c r="N48" s="41"/>
       <c r="O48" s="41"/>
-      <c r="P48" s="55"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="P48" s="133"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="47"/>
       <c r="E49" s="2"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -4220,6 +4217,140 @@
     </row>
   </sheetData>
   <mergeCells count="158">
+    <mergeCell ref="T46:U46"/>
+    <mergeCell ref="V46:W46"/>
+    <mergeCell ref="X46:Y46"/>
+    <mergeCell ref="Z46:AA46"/>
+    <mergeCell ref="AB46:AC46"/>
+    <mergeCell ref="AD46:AE46"/>
+    <mergeCell ref="T45:U45"/>
+    <mergeCell ref="V45:W45"/>
+    <mergeCell ref="X45:Y45"/>
+    <mergeCell ref="Z45:AA45"/>
+    <mergeCell ref="AB45:AC45"/>
+    <mergeCell ref="AD45:AE45"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="Q41:Q44"/>
+    <mergeCell ref="P45:P48"/>
+    <mergeCell ref="A30:A36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="AD39:AE39"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="V28:W28"/>
+    <mergeCell ref="X28:Y28"/>
+    <mergeCell ref="Z28:AA28"/>
+    <mergeCell ref="AB28:AC28"/>
+    <mergeCell ref="AD28:AE28"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="AB39:AC39"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="R45:S45"/>
+    <mergeCell ref="R46:S46"/>
+    <mergeCell ref="AF39:AF40"/>
+    <mergeCell ref="R41:S41"/>
+    <mergeCell ref="R42:S42"/>
+    <mergeCell ref="R43:S43"/>
+    <mergeCell ref="R44:S44"/>
+    <mergeCell ref="A37:P39"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:C41"/>
+    <mergeCell ref="P40:P41"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="Q39:Q40"/>
+    <mergeCell ref="R39:S40"/>
+    <mergeCell ref="T39:U39"/>
+    <mergeCell ref="V39:W39"/>
+    <mergeCell ref="X39:Y39"/>
+    <mergeCell ref="Z39:AA39"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="A5:P5"/>
+    <mergeCell ref="Q5:AE5"/>
+    <mergeCell ref="Q6:AE6"/>
+    <mergeCell ref="Q7:V7"/>
+    <mergeCell ref="W7:AD7"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="Q10:Q12"/>
+    <mergeCell ref="R10:S10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="R11:S11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="R12:S12"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:C9"/>
+    <mergeCell ref="AE7:AF7"/>
+    <mergeCell ref="L7:P7"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="AF8:AF9"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="V8:W8"/>
+    <mergeCell ref="X8:Y8"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="AB8:AC8"/>
+    <mergeCell ref="AD8:AE8"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:S9"/>
+    <mergeCell ref="A13:AF13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:C15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="R14:S15"/>
+    <mergeCell ref="AF14:AF15"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="T14:U14"/>
+    <mergeCell ref="V14:W14"/>
+    <mergeCell ref="X14:Y14"/>
+    <mergeCell ref="Z14:AA14"/>
+    <mergeCell ref="AB14:AC14"/>
+    <mergeCell ref="AD14:AE14"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="Q25:AF27"/>
+    <mergeCell ref="A27:P27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A16:A26"/>
+    <mergeCell ref="Q16:Q24"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="A1:Z4"/>
     <mergeCell ref="AA1:AF1"/>
     <mergeCell ref="AA2:AE4"/>
@@ -4244,144 +4375,10 @@
     <mergeCell ref="B28:C29"/>
     <mergeCell ref="P28:P29"/>
     <mergeCell ref="R20:S20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="Q25:AF27"/>
-    <mergeCell ref="A27:P27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A16:A26"/>
-    <mergeCell ref="Q16:Q24"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="A13:AF13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:C15"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="R14:S15"/>
-    <mergeCell ref="AF14:AF15"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="T14:U14"/>
-    <mergeCell ref="V14:W14"/>
-    <mergeCell ref="X14:Y14"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="AB14:AC14"/>
-    <mergeCell ref="AD14:AE14"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="X8:Y8"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="AB8:AC8"/>
-    <mergeCell ref="AD8:AE8"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:S9"/>
-    <mergeCell ref="C6:O6"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="Q5:AE5"/>
-    <mergeCell ref="Q6:AE6"/>
-    <mergeCell ref="Q7:V7"/>
-    <mergeCell ref="W7:AD7"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="Q10:Q12"/>
-    <mergeCell ref="R10:S10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="R11:S11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="R12:S12"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:C9"/>
-    <mergeCell ref="AE7:AF7"/>
-    <mergeCell ref="L7:P7"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="AF39:AF40"/>
-    <mergeCell ref="R41:S41"/>
-    <mergeCell ref="R42:S42"/>
-    <mergeCell ref="R43:S43"/>
-    <mergeCell ref="R44:S44"/>
-    <mergeCell ref="A37:P39"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:C41"/>
-    <mergeCell ref="P40:P41"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="Q39:Q40"/>
-    <mergeCell ref="R39:S40"/>
-    <mergeCell ref="T39:U39"/>
-    <mergeCell ref="V39:W39"/>
-    <mergeCell ref="X39:Y39"/>
-    <mergeCell ref="Z39:AA39"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="Q41:Q44"/>
-    <mergeCell ref="P45:P48"/>
-    <mergeCell ref="A30:A36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="AD39:AE39"/>
-    <mergeCell ref="T28:U28"/>
-    <mergeCell ref="V28:W28"/>
-    <mergeCell ref="X28:Y28"/>
-    <mergeCell ref="Z28:AA28"/>
-    <mergeCell ref="AB28:AC28"/>
-    <mergeCell ref="AD28:AE28"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="AB39:AC39"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="R45:S45"/>
-    <mergeCell ref="R46:S46"/>
-    <mergeCell ref="T46:U46"/>
-    <mergeCell ref="V46:W46"/>
-    <mergeCell ref="X46:Y46"/>
-    <mergeCell ref="Z46:AA46"/>
-    <mergeCell ref="AB46:AC46"/>
-    <mergeCell ref="AD46:AE46"/>
-    <mergeCell ref="T45:U45"/>
-    <mergeCell ref="V45:W45"/>
-    <mergeCell ref="X45:Y45"/>
-    <mergeCell ref="Z45:AA45"/>
-    <mergeCell ref="AB45:AC45"/>
-    <mergeCell ref="AD45:AE45"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.51181102362204722" top="0.31496062992125984" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="49" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="47" orientation="landscape" r:id="rId1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="32" max="1048575" man="1"/>
   </colBreaks>
@@ -4392,21 +4389,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="140" t="s">
         <v>69</v>
       </c>
       <c r="B1" s="140"/>
       <c r="C1" s="140"/>
     </row>
-    <row r="2" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>64</v>
       </c>
@@ -4417,12 +4414,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="160.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="160.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
     </row>
-    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>67</v>
       </c>
@@ -4431,14 +4428,14 @@
       </c>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="1:3" ht="162.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="162.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C5" s="4"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>63</v>
       </c>
@@ -4461,13 +4458,13 @@
                 <xdr:col>15</xdr:col>
                 <xdr:colOff>533400</xdr:colOff>
                 <xdr:row>20</xdr:row>
-                <xdr:rowOff>180975</xdr:rowOff>
+                <xdr:rowOff>182880</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>17</xdr:col>
-                <xdr:colOff>466725</xdr:colOff>
+                <xdr:colOff>464820</xdr:colOff>
                 <xdr:row>31</xdr:row>
-                <xdr:rowOff>95250</xdr:rowOff>
+                <xdr:rowOff>99060</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -4484,15 +4481,15 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>47625</xdr:colOff>
+                <xdr:colOff>45720</xdr:colOff>
                 <xdr:row>2</xdr:row>
-                <xdr:rowOff>57150</xdr:rowOff>
+                <xdr:rowOff>60960</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>1400175</xdr:colOff>
+                <xdr:colOff>1402080</xdr:colOff>
                 <xdr:row>2</xdr:row>
-                <xdr:rowOff>2000250</xdr:rowOff>
+                <xdr:rowOff>2004060</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -4509,9 +4506,9 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>66675</xdr:colOff>
+                <xdr:colOff>68580</xdr:colOff>
                 <xdr:row>2</xdr:row>
-                <xdr:rowOff>104775</xdr:rowOff>
+                <xdr:rowOff>106680</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
@@ -4534,15 +4531,15 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>95250</xdr:colOff>
+                <xdr:colOff>99060</xdr:colOff>
                 <xdr:row>4</xdr:row>
-                <xdr:rowOff>85725</xdr:rowOff>
+                <xdr:rowOff>83820</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>1419225</xdr:colOff>
+                <xdr:colOff>1417320</xdr:colOff>
                 <xdr:row>4</xdr:row>
-                <xdr:rowOff>2000250</xdr:rowOff>
+                <xdr:rowOff>2004060</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
@@ -4559,15 +4556,15 @@
             <anchor moveWithCells="1" sizeWithCells="1">
               <from>
                 <xdr:col>0</xdr:col>
-                <xdr:colOff>133350</xdr:colOff>
+                <xdr:colOff>137160</xdr:colOff>
                 <xdr:row>4</xdr:row>
-                <xdr:rowOff>47625</xdr:rowOff>
+                <xdr:rowOff>45720</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>0</xdr:col>
                 <xdr:colOff>1485900</xdr:colOff>
                 <xdr:row>4</xdr:row>
-                <xdr:rowOff>2000250</xdr:rowOff>
+                <xdr:rowOff>2004060</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>

</xml_diff>